<commit_message>
Rename to Modular Robot and add Pollen Robotics open-source files
- Remove every OreVis mention from the sandbox, physics bench, docs and v2
  workbook (title, robot speech, JS globals, storage keys, MJCF names).
- third_party/pollen: Pollen Robotics' Amazing Hand Python/Arduino examples and
  MuJoCo models (Apache 2.0, CC BY 4.0 meshes), unchanged, with NOTICE.md.
- third_party/fetch_pollen.sh: pinned download of the full AmazingHand repo
  (STL/STEP print files) and the Reachy Mini SDK and conversation app.
- sim/amazing_hand.py: runs Pollen's hand model through their named poses and
  reports the thumb-to-finger gaps.
- Plan v2 and the review now point the hand and voice stages at Pollen's code.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Urr7htkHCVGaVsVi8Qg9Un
</commit_message>
<xml_diff>
--- a/plan/robot_project_plan_v2.xlsx
+++ b/plan/robot_project_plan_v2.xlsx
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -805,7 +805,7 @@
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Stage 3 = build the duck's legs and put the OreVis shell, face and camera on top. Keep added mass under about 150 g. See sim/OPEN_DUCK.md</t>
+          <t>Stage 3 = build the duck's legs and put the round robot shell, face and camera on top. Keep added mass under about 150 g. See sim/OPEN_DUCK.md</t>
         </is>
       </c>
     </row>
@@ -883,59 +883,103 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>Software: write behaviours once, run them in the twin and on the robot</t>
+          <t>Use Pollen Robotics' open-source Amazing Hand files</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Give motors, servos and sensors the same small interface in the sandbox, MuJoCo and the robot. Tested behaviour code can then move to hardware unchanged.</t>
+          <t>Pollen publish the hand's print files (CC BY 4.0), servo code and a MuJoCo model (Apache 2.0). A copy is in third_party/pollen; python sim/amazing_hand.py runs their model through their named poses. Closed, the fingertips stop about 46 mm from the thumb, so tip-to-tip it can't pinch the 30 mm test blocks.</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>New software row 10: hal.py</t>
+          <t>Use their files as-is for the bench-mounted hand; test with 50 mm objects first</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Adapt</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>P04 does not need to wait for parts (P03)</t>
+          <t>Stage 5 voice: start from Pollen's Reachy Mini conversation app</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>The computer, Thonny and the sandbox can all be set up while parts ship.</t>
+          <t>Reachy Mini's SDK and conversation app are open source (Apache 2.0) and already connect a microphone, a speaker and a language model to a small robot.</t>
         </is>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>P04 dependency changed to None</t>
+          <t>third_party/fetch_pollen.sh downloads it; adapt its voice loop for P30-P31</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
         <is>
+          <t>Adapt</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Software: write behaviours once, run them in the twin and on the robot</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Give motors, servos and sensors the same small interface in the sandbox, MuJoCo and the robot. Tested behaviour code can then move to hardware unchanged.</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>New software row 10: hal.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
           <t>Fix</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>P04 does not need to wait for parts (P03)</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>The computer, Thonny and the sandbox can all be set up while parts ship.</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>P04 dependency changed to None</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>P18 live video now has a home</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Stage 2 adds the Pi Zero 2 W, which streams the camera. The Pico keeps doing motors and the face.</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>P18 linked to stage 2 tasks</t>
         </is>
@@ -1891,7 +1935,7 @@
       </c>
       <c r="B38" s="22" t="inlineStr">
         <is>
-          <t>Stage 3: OreVis head on the duck</t>
+          <t>Stage 3: robot head on the duck</t>
         </is>
       </c>
       <c r="C38" s="22" t="inlineStr">
@@ -2321,7 +2365,7 @@
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>Grows legs: Open Duck Mini v2 legs (10x STS3215), BNO055 IMU, 2S battery. OreVis shell becomes the head and body.</t>
+          <t>Grows legs: Open Duck Mini v2 legs (10x STS3215), BNO055 IMU, 2S battery. The round robot shell becomes the head and body.</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr">
@@ -3930,12 +3974,12 @@
       </c>
       <c r="B38" s="22" t="inlineStr">
         <is>
-          <t>Pollen Amazing Hand kit (optional)</t>
+          <t>Pollen Amazing Hand (optional): 8x Feetech SCS0009 + printed parts</t>
         </is>
       </c>
       <c r="C38" s="22" t="inlineStr">
         <is>
-          <t>8 servos, about 400 g. Too heavy for the walker; use on a bench arm.</t>
+          <t>Free print files and code from Pollen (third_party/pollen). About 400 g: too heavy for the walker, use on a bench arm.</t>
         </is>
       </c>
       <c r="D38" s="23" t="n">
@@ -3950,7 +3994,7 @@
       </c>
       <c r="G38" s="22" t="inlineStr">
         <is>
-          <t>https://huggingface.co/blog/pollen-robotics/amazing-hand</t>
+          <t>https://github.com/pollen-robotics/AmazingHand</t>
         </is>
       </c>
       <c r="H38" s="22" t="inlineStr">
@@ -4564,7 +4608,7 @@
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>Wake word, then speech-to-text, then the same command parser as the sandbox. Say 'stop' always wins.</t>
+          <t>Start from Pollen's Reachy Mini conversation app (third_party/fetch_pollen.sh). Speech goes to the same command parser as the sandbox. 'Stop' always wins.</t>
         </is>
       </c>
       <c r="E18" s="22" t="inlineStr">
@@ -4574,7 +4618,7 @@
       </c>
       <c r="F18" s="22" t="inlineStr">
         <is>
-          <t>https://github.com/rhasspy/piper</t>
+          <t>https://github.com/pollen-robotics/reachy_mini</t>
         </is>
       </c>
       <c r="G18" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Put Pollen's Amazing Hand into the sandbox
- sim/export_pollen_hand.py records Pollen's MuJoCo hand model (parts and
  finger linkages) moving from open to each of their demo poses; the sandbox
  plays the frames back (sandbox/pollen_hand.json + .bin, 1.6 MB).
- New Hand lab panel: pose buttons, finger travel, Pollen's demo sequence,
  live servo angles, and a button to fit the hand to the robot's arm.
- The Amazing Hand on the robot uses the real model; "hand <pose>" program
  command and spoken poses ("make a fist", "point").
- Simulation now steps in small slices so it keeps real time when drawing
  is slow; the hand lab only renders while on screen.
- Amazing Hand length set to its real ~185 mm; bench and plan results updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Urr7htkHCVGaVsVi8Qg9Un
</commit_message>
<xml_diff>
--- a/plan/robot_project_plan_v2.xlsx
+++ b/plan/robot_project_plan_v2.xlsx
@@ -844,7 +844,7 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Pollen's Amazing Hand is about 400 g. The physics bench shows the 1.36 kg walker tips 44 degrees holding it out. A 45 g 3-finger tendon hand holds a 20 g block at 64% of shoulder stall with no tipping.</t>
+          <t>Pollen's Amazing Hand is about 400 g. The physics bench shows the 1.36 kg walker tips 37 degrees holding it out. A 45 g 3-finger tendon hand holds a 20 g block at 64% of shoulder stall with no tipping.</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
@@ -5581,7 +5581,7 @@
         </is>
       </c>
       <c r="J11" s="17" t="n">
-        <v>43.6</v>
+        <v>36.5</v>
       </c>
       <c r="K11" s="17" t="inlineStr">
         <is>

</xml_diff>